<commit_message>
Updated ScanResult and scan functions
</commit_message>
<xml_diff>
--- a/backend/cleaners.xlsx
+++ b/backend/cleaners.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac/Documents/source_codes/segp-g6/backend/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEGP-G6\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{821A7847-6135-8C4F-86B5-5ABFE099D847}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C778CF9-7A5F-4B5B-82F9-058D7EEFC8E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -57,11 +57,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -70,6 +70,13 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -117,7 +124,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -418,14 +425,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="19.375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="30.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -442,7 +449,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="112" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="148.5" x14ac:dyDescent="0.15">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -460,6 +467,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Clean data according to user respond
</commit_message>
<xml_diff>
--- a/backend/cleaners.xlsx
+++ b/backend/cleaners.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEGP-G6\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C778CF9-7A5F-4B5B-82F9-058D7EEFC8E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B394775-0E76-4857-90EC-8894A1D056ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12075" yWindow="1845" windowWidth="17085" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>fn_name</t>
   </si>
@@ -37,27 +37,123 @@
     <t>definition</t>
   </si>
   <si>
-    <t>remove_duplicates</t>
-  </si>
-  <si>
     <t>Duplicate Remover</t>
   </si>
   <si>
     <t>Removes duplicate entries.</t>
   </si>
   <si>
-    <t>def clean_df_for_duplicates(scan_result: ScanResult, df: pandas.DataFrame) -&gt; pandas.DataFrame:
+    <t>def clean_df_for_duplicates(scan_result: ScanResult, df: pd.DataFrame) -&gt; pd.DataFrame:
     for action in scan_result.actions:
-        if isinstance(action, ScanResultAction):
-            print(f"{action}")
+        if action.activate:
+            if action.cleaner == "remove":
+                df = df.drop_duplicates(keep='first')
+            elif action.cleaner == "keep":
+                pass
     return df</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>def clean_df_for_missing(scan_result: ScanResult, df: pd.DataFrame) -&gt; pd.DataFrame:
+    for action in scan_result.actions:
+        if action.activate:
+            col = scan_result.col
+            row_idx = scan_result.row
+            if row_idx not in df.index or col not in df.columns:
+                continue
+            if action.cleaner == "mean":
+                df.at[row_idx, col] = df[col].mean()
+            elif action.cleaner == "median":
+                df.at[row_idx, col] = df[col].median()
+            elif action.cleaner == "mode":
+                mode_val = df[col].mode()
+                if not mode_val.empty:
+                    df.at[row_idx, col] = mode_val.iloc[0]
+            elif action.cleaner == "ffill":
+                prev_valid = df.loc[:row_idx, col].dropna()
+                if not prev_valid.empty:
+                    df.at[row_idx, col] = prev_valid.iloc[-1]
+            elif action.cleaner == "bfill":
+                next_valid = df.loc[row_idx:, col].dropna()
+                if not next_valid.empty:
+                    df.at[row_idx, col] = next_valid.iloc[0]
+            elif action.cleaner == "delete":
+                df = df.drop(index=row_idx)
+    return df</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Missing Value Filler</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>def clean_df_for_outliers(scan_result: ScanResult, df: pd.DataFrame) -&gt; pd.DataFrame:
+    for action in scan_result.actions:
+        if action.activate:
+            if action.cleaner == "delete":
+                df = df.drop(index=scan_result.row)
+    return df</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Removes outlier rows</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fills in the missing values</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Outliers Remover</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>clean_df_for_duplicates</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>clean_df_for_missing</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>clean_df_for_outliers</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>clean_df_for_categorical</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Categorical features Encoder</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Encode categorical features</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>def clean_df_for_categorical(scan_result: ScanResult, df: pd.DataFrame) -&gt; pd.DataFrame:
+    for action in scan_result.actions:
+        if action.activate:
+            col = scan_result.col
+            if col not in df.columns:
+                continue
+            if action.cleaner == "one_hot":
+                dummies = pd.get_dummies(df[col], prefix=col)
+                df = pd.concat([df.drop(col, axis=1), dummies], axis=1)
+            elif action.cleaner == "label_encoding":
+                df[col] = df[col].astype('category').cat.codes
+            elif action.cleaner == "drop":
+                df = df.drop(col, axis=1)
+    return df</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -73,6 +169,14 @@
     </font>
     <font>
       <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <family val="3"/>
       <charset val="134"/>
@@ -114,7 +218,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -122,6 +226,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -424,10 +530,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="2" width="19.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="30.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="35.125" bestFit="1" customWidth="1"/>
   </cols>
@@ -449,25 +556,77 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="148.5" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:5" ht="202.5" x14ac:dyDescent="0.15">
       <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="409.5" x14ac:dyDescent="0.15">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="162" x14ac:dyDescent="0.15">
+      <c r="A4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="405" x14ac:dyDescent="0.15">
+      <c r="A5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update cleaners.xlsx and SRActionType
</commit_message>
<xml_diff>
--- a/backend/cleaners.xlsx
+++ b/backend/cleaners.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEGP-G6\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B394775-0E76-4857-90EC-8894A1D056ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90274921-87E8-4885-AD12-3C6EC972DD7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12075" yWindow="1845" windowWidth="17085" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4995" yWindow="2805" windowWidth="21600" windowHeight="11265" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t>fn_name</t>
   </si>
@@ -37,98 +37,361 @@
     <t>definition</t>
   </si>
   <si>
-    <t>Duplicate Remover</t>
-  </si>
-  <si>
-    <t>Removes duplicate entries.</t>
+    <t>clean_df_for_duplicates</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>clean_df_for_missing</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>clean_df_for_categorical</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Categorical features Encoder</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Encode categorical features</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>def scan_df_for_duplicates(df: pd.DataFrame) -&gt; List[ScanResult]:
+    scan_results = []
+    df = df.dropna(axis=1, how='all')
+    duplicated_rows = df[df.duplicated(keep="first")]
+    for index in duplicated_rows.index:
+        actions = [
+            ScanResultAction(
+                title="Duplication Remover",
+                description="Remove the duplicated rows",
+                cleaner="clean_df_for_duplicates",
+                cleaner_id= None,
+                activate=True
+            )
+        ]
+        scan_results.append(
+            ScanResult(
+                row=index,
+                col=-1,  # No specific column as the entire row is duplicated
+                message=f"Row {index + 1} is duplicated",
+                action_type=SRActionType.ONE_MANDATORY,
+                actions=actions
+            )
+        )
+    return scan_results</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>def scan_df_for_missing(df: pd.DataFrame) -&gt; List[ScanResult]:
+    missing_matrix = df.isna()
+    scan_results = []
+    for row_idx, col_idx in zip(*np.where(missing_matrix)):
+        col_name = df.columns[col_idx]
+        # Check if the column is numeric
+        if pd.api.types.is_numeric_dtype(df[col_name]):
+            actions = [
+                ScanResultAction(
+                    title="Missing Value Filler",
+                    description="Fill with mean value",
+                    cleaner="fill_with_mean",
+                    cleaner_id=None,
+                    activate=True
+                ),
+                ScanResultAction(
+                    title="Missing Value Filler",
+                    description="Fill with median value",
+                    cleaner="fill_with_median",
+                    cleaner_id=None,
+                    activate=True
+                ),
+                ScanResultAction(
+                    title="Missing Value Filler",
+                    description="Fill with most frequent value",
+                    cleaner="fill_with_mode",
+                    cleaner_id=None,
+                    activate=True
+                ),
+                ScanResultAction(
+                    title="Missing Value Filler",
+                    description="Fill with previous value",
+                    cleaner="fill_with_ffill",
+                    cleaner_id=None,
+                    activate=True
+                ),
+                ScanResultAction(
+                    title="Missing Value Filler",
+                    description="Fill with next value",
+                    cleaner="fill_with_bfill",
+                    cleaner_id=None,
+                    activate=True
+                ),
+                ScanResultAction(
+                    title="Missing Value Filler",
+                    description="Delete the row",
+                    cleaner="delete_missing_rows",
+                    cleaner_id=None,
+                    activate=True
+                )
+            ]
+        else:
+            # For non-numeric columns, offer only mode, ffill, bfill, and delete
+            actions = [
+                ScanResultAction(
+                    title="Missing Value Filler",
+                    description="Fill with most frequent value",
+                    cleaner="fill_with_mode",
+                    cleaner_id=None,
+                    activate=True
+                ),
+                ScanResultAction(
+                    title="Missing Value Filler",
+                    description="Fill with previous value",
+                    cleaner="fill_with_ffill",
+                    cleaner_id=None,
+                    activate=True
+                ),
+                ScanResultAction(
+                    title="Missing Value Filler",
+                    description="Fill with next value",
+                    cleaner="fill_with_bfill",
+                    cleaner_id=None,
+                    activate=True
+                ),
+                ScanResultAction(
+                    title="Missing Value Filler",
+                    description="Delete the row",
+                    cleaner="delete_missing_rows",
+                    cleaner_id=None,
+                    activate=True
+                )
+            ]
+        scan_results.append(
+            ScanResult(
+                row=row_idx,
+                col=col_name,
+                message=f"Missing value in row {row_idx+1}, column '{col_name}'",
+                action_type=SRActionType.ONE_MANDATORY,
+                actions=actions
+            )
+        )
+    return scan_results</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>scan_df_for_duplicates</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>scan_df_for_missing</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>scan_df_for_outliers</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>scan_df_for_categorical</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Duplicate Scanner</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Missing Value Scanner</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Outliers Scanner</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Categorical features Scanner</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Scan outlier rows</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Scan categorical features</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>def scan_df_for_categorical(df: pd.DataFrame) -&gt; List[ScanResult]:
+    scan_results = []
+    # max_categories = int(len(df) * 0.1)
+    categorical_dtypes: list = ['object', 'category', 'bool']
+    non_numeric_cols = df.select_dtypes(include=categorical_dtypes)
+    for col in non_numeric_cols.columns:
+        if df[col].dropna().size == 0:
+            continue
+        unique_count = df[col].nunique()
+        # if unique_count &gt; max_categories:
+        #     continue
+        categories = df[col].dropna().unique()
+        categories_str = ", ".join(map(str, categories[:10]))
+        if len(categories) &gt; 10:
+            categories_str += f"... (Total {len(categories)} categories)"
+        actions = [
+            ScanResultAction(
+                title="Categorical Encoder",
+                description="Apply one-hot encoding",
+                cleaner="one_hot",
+                cleaner_id=None,
+                activate=True
+            ),
+            ScanResultAction(
+                title="Categorical Encoder",
+                description="Apply label encoding",
+                cleaner="label_encoding",
+                cleaner_id=None,
+                activate=True
+            ),
+            ScanResultAction(
+                title="Categorical Encoder",
+                description="Drop the column",
+                cleaner="drop",
+                cleaner_id=None,
+                activate=True
+            )
+        ]
+        scan_results.append(
+            ScanResult(
+                row=-1,
+                col=col,
+                message=f"Categorical feature '{col}' detected with {unique_count} categories: {categories_str}",
+                action_type=SRActionType.ONE_MANDATORY,
+                actions=actions
+            )
+        )
+    return scan_results</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>def scan_df_for_outliers(df: pd.DataFrame) -&gt; List[ScanResult]:
+    scan_results = []
+    for col in df.select_dtypes(include=[np.number]):
+        col_data = df[col].dropna()
+        if col_data.empty:
+            continue
+        q1, q3 = col_data.quantile([0.25, 0.75])
+        iqr = q3 - q1
+        lower_bound = q1 - 1.5 * iqr
+        upper_bound = q3 + 1.5 * iqr
+        outliers = (col_data &lt; lower_bound) | (col_data &gt; upper_bound)
+        for idx in col_data[outliers].index:
+            actions = [
+                ScanResultAction(
+                    title="Outlier Handler",
+                    description="Delete the outlier",
+                    cleaner="delete_outlier",
+                    cleaner_id=None,
+                    activate=True
+                )
+            ]
+            scan_results.append(
+                ScanResult(
+                    row=idx,
+                    col=col,
+                    message=f"Outlier detected in column '{col}' at row {idx+1}",
+                    action_type=SRActionType.ONE_MANDATORY,
+                    actions=actions
+                )
+            )
+    return scan_results</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>def clean_df_for_duplicates(scan_result: ScanResult, df: pd.DataFrame) -&gt; pd.DataFrame:
     for action in scan_result.actions:
-        if action.activate:
-            if action.cleaner == "remove":
+        if action.cleaner == clean_df_for_duplicates.__name__:
+            if action.activate:
                 df = df.drop_duplicates(keep='first')
-            elif action.cleaner == "keep":
-                pass
     return df</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>def scan_df_for_target(df: pd.DataFrame, target) -&gt; List[ScanResult]:
+    scan_results = []
+    matches = df.isin([target])
+    for row_idx, col_idx in zip(*np.where(matches)):
+        col_name = df.columns[col_idx]
+        actions = [
+            ScanResultAction(
+                title=f"Handle '{target}' value",
+                description=f"Handle the '{target}' value in column '{col_name}'",
+                cleaner="handle_target",
+                activate=True,
+            ),
+            ScanResultAction(
+                title="Delete row",
+                description=f"Delete row {row_idx+1} because it contains '{target}'",
+                cleaner="delete_target_row",
+                activate=True,
+            ),
+            ScanResultAction(
+                title="Delete column",
+                description=f"Delete column '{col_name}' because it contains '{target}'",
+                cleaner="delete_target_column",
+                activate=True,
+            )
+        ]
+        scan_results.append(
+            ScanResult(
+                row=row_idx,
+                col=col_name,
+                message=f"Target value '{target}' found in row {row_idx+1}, column '{col_name}'",
+                action_type=SRActionType.MANY_OPTIONAL,
+                actions=actions
+            )
+        )
+    return scan_results</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>scan_df_for_target</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Target Scanner</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Scan for target element in the table</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>def clean_df_for_missing(scan_result: ScanResult, df: pd.DataFrame) -&gt; pd.DataFrame:
     for action in scan_result.actions:
         if action.activate:
-            col = scan_result.col
-            row_idx = scan_result.row
-            if row_idx not in df.index or col not in df.columns:
-                continue
-            if action.cleaner == "mean":
-                df.at[row_idx, col] = df[col].mean()
-            elif action.cleaner == "median":
-                df.at[row_idx, col] = df[col].median()
-            elif action.cleaner == "mode":
-                mode_val = df[col].mode()
-                if not mode_val.empty:
-                    df.at[row_idx, col] = mode_val.iloc[0]
-            elif action.cleaner == "ffill":
-                prev_valid = df.loc[:row_idx, col].dropna()
-                if not prev_valid.empty:
-                    df.at[row_idx, col] = prev_valid.iloc[-1]
-            elif action.cleaner == "bfill":
-                next_valid = df.loc[row_idx:, col].dropna()
-                if not next_valid.empty:
-                    df.at[row_idx, col] = next_valid.iloc[0]
-            elif action.cleaner == "delete":
-                df = df.drop(index=row_idx)
+            if action.cleaner == "fill_with_mean":
+                df[scan_result.col].fillna(df[scan_result.col].mean(), inplace=True)
+            elif action.cleaner == "fill_with_median":
+                df[scan_result.col].fillna(df[scan_result.col].median(), inplace=True)
+            elif action.cleaner == "fill_with_mode":
+                df[scan_result.col].fillna(df[scan_result.col].mode()[0], inplace=True)
+            elif action.cleaner == "fill_with_ffill":
+                df[scan_result.col].fillna(method='ffill', inplace=True)
+            elif action.cleaner == "fill_with_bfill":
+                df[scan_result.col].fillna(method='bfill', inplace=True)
+            elif action.cleaner == "delete_missing_rows":
+                df.dropna(subset=[scan_result.col], inplace=True)
     return df</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>Missing Value Filler</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>def clean_df_for_outliers(scan_result: ScanResult, df: pd.DataFrame) -&gt; pd.DataFrame:
+    <t>def clean_df_for_outlier(scan_result, df):
     for action in scan_result.actions:
         if action.activate:
-            if action.cleaner == "delete":
-                df = df.drop(index=scan_result.row)
+            if action.cleaner == "delete_outlier":
+                if scan_result.row in df.index:
+                    df.drop(index=scan_result.row, inplace=True)
+                else:
+                    print(f"Row {scan_result.row} not found in DataFrame.")
     return df</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Removes outlier rows</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Fills in the missing values</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Outliers Remover</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>clean_df_for_duplicates</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>clean_df_for_missing</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>clean_df_for_outliers</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>clean_df_for_categorical</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Categorical features Encoder</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Encode categorical features</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -146,6 +409,65 @@
             elif action.cleaner == "drop":
                 df = df.drop(col, axis=1)
     return df</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>def apply_target_cleaning(scan_result: ScanResult, df: pd.DataFrame) -&gt; pd.DataFrame:
+    for action in scan_result.actions:
+        if action.activate:
+            if action.cleaner == "delete_target_row":
+                df.drop(index=scan_result.row, inplace=True)
+            elif action.cleaner == "delete_target_column":
+                df.drop(columns=[scan_result.col], inplace=True)
+    return df</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>clean_df_for_outlier</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>apply_target_cleaning</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Apply target operation</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Remove the duplicate entries</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Scan duplicate entries</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Scan missing values</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fill in missing values</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Remove outliers</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Duplicate Remover</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Missing values Filler</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>outliers Remover</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Apply target operation on rows or columns</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -530,16 +852,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="26.125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="35.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -556,72 +878,174 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="202.5" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>37</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="409.5" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="162" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="405" x14ac:dyDescent="0.15">
-      <c r="A5" s="4" t="s">
-        <v>17</v>
+    <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A5" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A7" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A8" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A9" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A10" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A11" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>